<commit_message>
Rebuild site for v2.55
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMEqc6TnzEK4sWnwQy9Js9
</commit_message>
<xml_diff>
--- a/25_Templates/AI_Security_Audit_and_Evidence_Checklist.xlsx
+++ b/25_Templates/AI_Security_Audit_and_Evidence_Checklist.xlsx
@@ -41,7 +41,7 @@
     <t xml:space="preserve">AI Security Audit and Evidence Checklist</t>
   </si>
   <si>
-    <t xml:space="preserve">Built from the AI Security Wiki (https://nachi065.github.io/AI-Security-Wiki/) on 29 October 2026. Version 1.3.</t>
+    <t xml:space="preserve">Built from the AI Security Wiki (https://nachi065.github.io/AI-Security-Wiki/) on 29 October 2026. Version 1.4.</t>
   </si>
   <si>
     <t xml:space="preserve">Read first</t>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">AI Security Audit and Evidence Checklist Copyright (c) 2026 Nachiket Sathaye and Ankush Jain. Licensed under CC BY-SA 4.0 (https://creativecommons.org/licenses/by-sa/4.0/). See the License sheet for credit, ShareAlike and third-party terms.</t>
   </si>
   <si>
-    <t xml:space="preserve">AI Security Audit and Evidence Checklist, version 1.3, 29 October 2026</t>
+    <t xml:space="preserve">AI Security Audit and Evidence Checklist, version 1.4, 29 October 2026</t>
   </si>
   <si>
     <t xml:space="preserve">License notice</t>

</xml_diff>

<commit_message>
Rebuild site for v2.56
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TMEqc6o8aawa4eKgvtuFZz
</commit_message>
<xml_diff>
--- a/25_Templates/AI_Security_Audit_and_Evidence_Checklist.xlsx
+++ b/25_Templates/AI_Security_Audit_and_Evidence_Checklist.xlsx
@@ -41,7 +41,7 @@
     <t xml:space="preserve">AI Security Audit and Evidence Checklist</t>
   </si>
   <si>
-    <t xml:space="preserve">Built from the AI Security Wiki (https://nachi065.github.io/AI-Security-Wiki/) on 29 October 2026. Version 1.4.</t>
+    <t xml:space="preserve">Built from the AI Security Wiki (https://nachi065.github.io/AI-Security-Wiki/) on 29 October 2026. Version 1.5.</t>
   </si>
   <si>
     <t xml:space="preserve">Read first</t>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">AI Security Audit and Evidence Checklist Copyright (c) 2026 Nachiket Sathaye and Ankush Jain. Licensed under CC BY-SA 4.0 (https://creativecommons.org/licenses/by-sa/4.0/). See the License sheet for credit, ShareAlike and third-party terms.</t>
   </si>
   <si>
-    <t xml:space="preserve">AI Security Audit and Evidence Checklist, version 1.4, 29 October 2026</t>
+    <t xml:space="preserve">AI Security Audit and Evidence Checklist, version 1.5, 29 October 2026</t>
   </si>
   <si>
     <t xml:space="preserve">License notice</t>
@@ -839,7 +839,7 @@
     <t xml:space="preserve">AI Policy, Roles and Acceptable Use</t>
   </si>
   <si>
-    <t xml:space="preserve">Approved policy; board-approved AI strategy and risk appetite with its review record; roles and responsibilities record; governance decision log; policy-to-control mapping; training and acknowledgement records.</t>
+    <t xml:space="preserve">Approved policy; board-approved AI strategy and risk appetite with its review record; roles and responsibilities record; governance decision log; policy-to-control mapping; training and acknowledgement records; policy alignment record; employment and contractor terms covering AI use.</t>
   </si>
   <si>
     <t xml:space="preserve">Select policy statements and trace each to a control and to evidence that it operates. Confirm the policy was reviewed within its cycle.</t>
@@ -875,7 +875,7 @@
     <t xml:space="preserve">Third-Party and Vendor AI Assurance</t>
   </si>
   <si>
-    <t xml:space="preserve">Vendor assessments; contract clauses; sub-processor list; model change notices.</t>
+    <t xml:space="preserve">Vendor assessments; contract clauses; sub-processor list; model change notices; exit return or deletion confirmation.</t>
   </si>
   <si>
     <t xml:space="preserve">Sample AI vendors in use and confirm each has a current assessment and the required contract terms. Confirm the last model or terms change triggered a review.</t>
@@ -1154,7 +1154,7 @@
     <t xml:space="preserve">Assurance and Testing</t>
   </si>
   <si>
-    <t xml:space="preserve">Threat models; architecture review records; control selection; approvals and exceptions.</t>
+    <t xml:space="preserve">Threat models; architecture review records; control selection; approvals and exceptions; responsible development objectives.</t>
   </si>
   <si>
     <t xml:space="preserve">Sample production systems and confirm each has a current threat model, a control selection that matches its tier and a signed approval.</t>
@@ -1169,7 +1169,7 @@
     <t xml:space="preserve">Adversarial Testing and Continuous Evaluation</t>
   </si>
   <si>
-    <t xml:space="preserve">Red team reports; regression suite results; agreed thresholds; retest records.</t>
+    <t xml:space="preserve">Red team reports; regression suite results; agreed thresholds; retest records; threat intelligence review log; production test authorisations.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm the last model or prompt change triggered the regression suite. Reproduce a sample of reported findings and confirm fixes hold.</t>
@@ -6867,7 +6867,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="41" t="s">
         <v>265</v>
       </c>
@@ -8143,7 +8143,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="41" t="s">
         <v>375</v>
       </c>

</xml_diff>